<commit_message>
chore(guide): 配表新增 GuideOverlayClicked 触发器实例并重导 config.db
Guide.xlsx/trigger_ref 加一行可复用实例(420003, TypeId=2100, PayloadId=0)，
对话步骤把 CompleteTriggerId 指向它即"点任意处继续"。重导同步首包/热更两个
config.db 与 GuideIds.g.cs 常量。未新增 payload 表——避免又一个 >31 字符表名
(Excel 打开必修复的既有毛病，表名即 table 名不可改)。CI 全绿。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assets/RefData_Excel/Guide.xlsx
+++ b/Assets/RefData_Excel/Guide.xlsx
@@ -2706,7 +2706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2836,6 +2836,27 @@
       <c r="E5" s="41" t="inlineStr">
         <is>
           <t>点击领取金币按钮完成步骤</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="71" t="n">
+        <v>420003</v>
+      </c>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>GuideOverlayClicked</t>
+        </is>
+      </c>
+      <c r="C6" s="72" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D6" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>孔外压暗区被点击/点任意处继续：对话步骤把 CompleteTriggerId 指向此行（无参，PayloadId 忽略）</t>
         </is>
       </c>
     </row>

</xml_diff>